<commit_message>
atualizei os dados do 3Q26 da AAPL
</commit_message>
<xml_diff>
--- a/analise_eua/tecnologia/apple/aapl_indicators.xlsx
+++ b/analise_eua/tecnologia/apple/aapl_indicators.xlsx
@@ -592,10 +592,10 @@
         <v>2025</v>
       </c>
       <c r="B2" t="n">
-        <v>33.92</v>
+        <v>33.89</v>
       </c>
       <c r="C2" t="n">
-        <v>33.93</v>
+        <v>33.9</v>
       </c>
       <c r="D2" t="n">
         <v>2.95</v>
@@ -607,10 +607,10 @@
         <v>26.92</v>
       </c>
       <c r="G2" t="n">
-        <v>51.55</v>
+        <v>51.5</v>
       </c>
       <c r="H2" t="n">
-        <v>3799161275</v>
+        <v>3795573635</v>
       </c>
       <c r="I2" t="n">
         <v>112377</v>
@@ -628,7 +628,7 @@
         <v>-0.27</v>
       </c>
       <c r="N2" t="n">
-        <v>26.39</v>
+        <v>26.36</v>
       </c>
       <c r="O2" t="n">
         <v>151.91</v>
@@ -687,10 +687,10 @@
         <v>2024</v>
       </c>
       <c r="B3" t="n">
-        <v>37.89</v>
+        <v>37.86</v>
       </c>
       <c r="C3" t="n">
-        <v>37.89</v>
+        <v>37.85</v>
       </c>
       <c r="D3" t="n">
         <v>2.64</v>
@@ -702,10 +702,10 @@
         <v>23.97</v>
       </c>
       <c r="G3" t="n">
-        <v>62.39</v>
+        <v>62.34</v>
       </c>
       <c r="H3" t="n">
-        <v>3551778888.84</v>
+        <v>3548556694.41</v>
       </c>
       <c r="I3" t="n">
         <v>119059</v>
@@ -723,7 +723,7 @@
         <v>-0.66</v>
       </c>
       <c r="N3" t="n">
-        <v>26.65</v>
+        <v>26.63</v>
       </c>
       <c r="O3" t="n">
         <v>164.59</v>
@@ -782,10 +782,10 @@
         <v>2023</v>
       </c>
       <c r="B4" t="n">
-        <v>27.47</v>
+        <v>27.44</v>
       </c>
       <c r="C4" t="n">
-        <v>27.47</v>
+        <v>27.45</v>
       </c>
       <c r="D4" t="n">
         <v>3.64</v>
@@ -797,10 +797,10 @@
         <v>25.31</v>
       </c>
       <c r="G4" t="n">
-        <v>42.84</v>
+        <v>42.8</v>
       </c>
       <c r="H4" t="n">
-        <v>2664396212.13</v>
+        <v>2661877135.17</v>
       </c>
       <c r="I4" t="n">
         <v>123930</v>
@@ -818,7 +818,7 @@
         <v>-0.61</v>
       </c>
       <c r="N4" t="n">
-        <v>21.48</v>
+        <v>21.46</v>
       </c>
       <c r="O4" t="n">
         <v>156.08</v>
@@ -877,10 +877,10 @@
         <v>2022</v>
       </c>
       <c r="B5" t="n">
+        <v>22.04</v>
+      </c>
+      <c r="C5" t="n">
         <v>22.06</v>
-      </c>
-      <c r="C5" t="n">
-        <v>22.08</v>
       </c>
       <c r="D5" t="n">
         <v>4.53</v>
@@ -892,10 +892,10 @@
         <v>25.31</v>
       </c>
       <c r="G5" t="n">
-        <v>43.52</v>
+        <v>43.48</v>
       </c>
       <c r="H5" t="n">
-        <v>2201965615.77</v>
+        <v>2200019700.21</v>
       </c>
       <c r="I5" t="n">
         <v>132480</v>
@@ -913,7 +913,7 @@
         <v>-0.72</v>
       </c>
       <c r="N5" t="n">
-        <v>17.15</v>
+        <v>17.13</v>
       </c>
       <c r="O5" t="n">
         <v>196.96</v>
@@ -972,10 +972,10 @@
         <v>2021</v>
       </c>
       <c r="B6" t="n">
-        <v>24.39</v>
+        <v>24.37</v>
       </c>
       <c r="C6" t="n">
-        <v>24.38</v>
+        <v>24.36</v>
       </c>
       <c r="D6" t="n">
         <v>4.1</v>
@@ -987,10 +987,10 @@
         <v>25.88</v>
       </c>
       <c r="G6" t="n">
-        <v>36.58</v>
+        <v>36.54</v>
       </c>
       <c r="H6" t="n">
-        <v>2309117866.72</v>
+        <v>2306946701.36</v>
       </c>
       <c r="I6" t="n">
         <v>136522</v>
@@ -1008,7 +1008,7 @@
         <v>-0.86</v>
       </c>
       <c r="N6" t="n">
-        <v>19.65</v>
+        <v>19.64</v>
       </c>
       <c r="O6" t="n">
         <v>150.07</v>
@@ -1067,13 +1067,13 @@
         <v>2020</v>
       </c>
       <c r="B7" t="n">
-        <v>33.98</v>
+        <v>33.95</v>
       </c>
       <c r="C7" t="n">
-        <v>33.97</v>
+        <v>33.94</v>
       </c>
       <c r="D7" t="n">
-        <v>2.94</v>
+        <v>2.95</v>
       </c>
       <c r="E7" t="n">
         <v>77344</v>
@@ -1082,10 +1082,10 @@
         <v>20.91</v>
       </c>
       <c r="G7" t="n">
-        <v>29.82</v>
+        <v>29.8</v>
       </c>
       <c r="H7" t="n">
-        <v>1951072260.36</v>
+        <v>1949163527.27</v>
       </c>
       <c r="I7" t="n">
         <v>122278</v>
@@ -1103,7 +1103,7 @@
         <v>-1.06</v>
       </c>
       <c r="N7" t="n">
-        <v>26.13</v>
+        <v>26.1</v>
       </c>
       <c r="O7" t="n">
         <v>87.87</v>
@@ -1162,10 +1162,10 @@
         <v>2019</v>
       </c>
       <c r="B8" t="n">
-        <v>17.99</v>
+        <v>17.98</v>
       </c>
       <c r="C8" t="n">
-        <v>17.99</v>
+        <v>17.97</v>
       </c>
       <c r="D8" t="n">
         <v>5.56</v>
@@ -1177,10 +1177,10 @@
         <v>21.24</v>
       </c>
       <c r="G8" t="n">
-        <v>10.99</v>
+        <v>10.98</v>
       </c>
       <c r="H8" t="n">
-        <v>994312016.88</v>
+        <v>993388450.08</v>
       </c>
       <c r="I8" t="n">
         <v>118885</v>
@@ -1198,7 +1198,7 @@
         <v>-0.96</v>
       </c>
       <c r="N8" t="n">
-        <v>14.14</v>
+        <v>14.13</v>
       </c>
       <c r="O8" t="n">
         <v>61.06</v>
@@ -1257,13 +1257,13 @@
         <v>2018</v>
       </c>
       <c r="B9" t="n">
-        <v>17.79</v>
+        <v>17.77</v>
       </c>
       <c r="C9" t="n">
-        <v>17.79</v>
+        <v>17.78</v>
       </c>
       <c r="D9" t="n">
-        <v>5.62</v>
+        <v>5.63</v>
       </c>
       <c r="E9" t="n">
         <v>81801</v>
@@ -1272,10 +1272,10 @@
         <v>22.41</v>
       </c>
       <c r="G9" t="n">
-        <v>9.880000000000001</v>
+        <v>9.869999999999999</v>
       </c>
       <c r="H9" t="n">
-        <v>1058864957.36</v>
+        <v>1057873881.96</v>
       </c>
       <c r="I9" t="n">
         <v>124110</v>
@@ -1293,7 +1293,7 @@
         <v>-1.05</v>
       </c>
       <c r="N9" t="n">
-        <v>14.33</v>
+        <v>14.31</v>
       </c>
       <c r="O9" t="n">
         <v>55.56</v>
@@ -1352,13 +1352,13 @@
         <v>2017</v>
       </c>
       <c r="B10" t="n">
-        <v>15.51</v>
+        <v>15.49</v>
       </c>
       <c r="C10" t="n">
-        <v>15.5</v>
+        <v>15.49</v>
       </c>
       <c r="D10" t="n">
-        <v>6.45</v>
+        <v>6.46</v>
       </c>
       <c r="E10" t="n">
         <v>71501</v>
@@ -1370,7 +1370,7 @@
         <v>5.59</v>
       </c>
       <c r="H10" t="n">
-        <v>749822020.24</v>
+        <v>749195951.1999999</v>
       </c>
       <c r="I10" t="n">
         <v>125225</v>
@@ -1388,7 +1388,7 @@
         <v>-1.07</v>
       </c>
       <c r="N10" t="n">
-        <v>12.5</v>
+        <v>12.49</v>
       </c>
       <c r="O10" t="n">
         <v>36.07</v>
@@ -1453,7 +1453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE18"/>
+  <dimension ref="A1:AE19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1610,1616 +1610,1711 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
-        <v>46109</v>
+        <v>46200</v>
       </c>
       <c r="B2" t="n">
-        <v>125.9</v>
+        <v>142.36</v>
       </c>
       <c r="C2" t="n">
-        <v>31.37</v>
+        <v>34.16</v>
       </c>
       <c r="D2" t="n">
-        <v>3.19</v>
+        <v>2.93</v>
       </c>
       <c r="E2" t="n">
-        <v>39324</v>
+        <v>39015</v>
       </c>
       <c r="F2" t="n">
-        <v>26.6</v>
+        <v>27.23</v>
       </c>
       <c r="G2" t="n">
-        <v>34.96</v>
+        <v>39.42</v>
       </c>
       <c r="H2" t="n">
-        <v>3723931223.62</v>
+        <v>4240891989.6</v>
       </c>
       <c r="I2" t="n">
-        <v>84711</v>
+        <v>84344</v>
       </c>
       <c r="J2" t="n">
-        <v>146595</v>
+        <v>146517</v>
       </c>
       <c r="K2" t="n">
-        <v>-61884</v>
+        <v>-62173</v>
       </c>
       <c r="L2" t="n">
-        <v>-0.39</v>
+        <v>-0.38</v>
       </c>
       <c r="M2" t="n">
         <v>-0.58</v>
       </c>
       <c r="N2" t="n">
-        <v>24.16</v>
+        <v>26.33</v>
       </c>
       <c r="O2" t="n">
-        <v>112.58</v>
+        <v>116.16</v>
       </c>
       <c r="P2" t="n">
-        <v>62.89</v>
+        <v>64.84</v>
       </c>
       <c r="Q2" t="n">
-        <v>28702</v>
+        <v>34369</v>
       </c>
       <c r="R2" t="n">
-        <v>-6168</v>
+        <v>-7757</v>
       </c>
       <c r="S2" t="n">
-        <v>-22279</v>
+        <v>-32640</v>
       </c>
       <c r="T2" t="n">
-        <v>26731</v>
+        <v>31914</v>
       </c>
       <c r="U2" t="n">
-        <v>1971</v>
+        <v>2455</v>
       </c>
       <c r="V2" t="n">
-        <v>-1267</v>
+        <v>-2542</v>
       </c>
       <c r="W2" t="n">
-        <v>11419</v>
+        <v>11729</v>
       </c>
       <c r="X2" t="n">
-        <v>38455</v>
+        <v>40359</v>
       </c>
       <c r="Y2" t="n">
-        <v>9473</v>
+        <v>492</v>
       </c>
       <c r="Z2" t="n">
-        <v>37.52</v>
+        <v>33.91</v>
       </c>
       <c r="AA2" t="n">
-        <v>104364</v>
+        <v>114273</v>
       </c>
       <c r="AB2" t="n">
-        <v>113912</v>
+        <v>124449</v>
       </c>
       <c r="AC2" t="n">
-        <v>0.26</v>
+        <v>0.28</v>
       </c>
       <c r="AD2" t="n">
-        <v>12.92</v>
+        <v>13.55</v>
       </c>
       <c r="AE2" t="n">
-        <v>12288</v>
+        <v>25105</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>46018</v>
+        <v>46109</v>
       </c>
       <c r="B3" t="n">
-        <v>71.66</v>
+        <v>125.79</v>
       </c>
       <c r="C3" t="n">
-        <v>24.12</v>
+        <v>31.34</v>
       </c>
       <c r="D3" t="n">
-        <v>4.15</v>
+        <v>3.19</v>
       </c>
       <c r="E3" t="n">
-        <v>54066</v>
+        <v>39324</v>
       </c>
       <c r="F3" t="n">
-        <v>29.28</v>
+        <v>26.6</v>
       </c>
       <c r="G3" t="n">
-        <v>34.21</v>
+        <v>34.93</v>
       </c>
       <c r="H3" t="n">
-        <v>3016735718.9</v>
+        <v>3720556369.68</v>
       </c>
       <c r="I3" t="n">
-        <v>90509</v>
+        <v>84711</v>
       </c>
       <c r="J3" t="n">
-        <v>144795</v>
+        <v>146595</v>
       </c>
       <c r="K3" t="n">
-        <v>-54286</v>
+        <v>-61884</v>
       </c>
       <c r="L3" t="n">
-        <v>-0.33</v>
+        <v>-0.39</v>
       </c>
       <c r="M3" t="n">
-        <v>-0.62</v>
+        <v>-0.58</v>
       </c>
       <c r="N3" t="n">
-        <v>18.81</v>
+        <v>24.14</v>
       </c>
       <c r="O3" t="n">
-        <v>143.6</v>
+        <v>112.58</v>
       </c>
       <c r="P3" t="n">
-        <v>71.17</v>
+        <v>62.89</v>
       </c>
       <c r="Q3" t="n">
-        <v>53925</v>
+        <v>28702</v>
       </c>
       <c r="R3" t="n">
-        <v>-4886</v>
+        <v>-6168</v>
       </c>
       <c r="S3" t="n">
-        <v>-39656</v>
+        <v>-22279</v>
       </c>
       <c r="T3" t="n">
-        <v>51552</v>
+        <v>26731</v>
       </c>
       <c r="U3" t="n">
-        <v>2373</v>
+        <v>1971</v>
       </c>
       <c r="V3" t="n">
-        <v>61</v>
+        <v>-1267</v>
       </c>
       <c r="W3" t="n">
-        <v>10887</v>
+        <v>11419</v>
       </c>
       <c r="X3" t="n">
-        <v>36632</v>
+        <v>38455</v>
       </c>
       <c r="Y3" t="n">
-        <v>-4263</v>
+        <v>9473</v>
       </c>
       <c r="Z3" t="n">
-        <v>24.44</v>
+        <v>37.52</v>
       </c>
       <c r="AA3" t="n">
-        <v>118788</v>
+        <v>104364</v>
       </c>
       <c r="AB3" t="n">
-        <v>130514</v>
+        <v>113912</v>
       </c>
       <c r="AC3" t="n">
-        <v>0.27</v>
+        <v>0.26</v>
       </c>
       <c r="AD3" t="n">
-        <v>9.31</v>
+        <v>12.92</v>
       </c>
       <c r="AE3" t="n">
-        <v>24701</v>
+        <v>12288</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>45836</v>
+        <v>46018</v>
       </c>
       <c r="B4" t="n">
-        <v>140.65</v>
+        <v>71.59</v>
       </c>
       <c r="C4" t="n">
-        <v>31.46</v>
+        <v>24.1</v>
       </c>
       <c r="D4" t="n">
-        <v>3.18</v>
+        <v>4.15</v>
       </c>
       <c r="E4" t="n">
-        <v>31032</v>
+        <v>54066</v>
       </c>
       <c r="F4" t="n">
-        <v>24.92</v>
+        <v>29.28</v>
       </c>
       <c r="G4" t="n">
-        <v>50.04</v>
+        <v>34.17</v>
       </c>
       <c r="H4" t="n">
-        <v>3296071296.62</v>
+        <v>3013933568.88</v>
       </c>
       <c r="I4" t="n">
-        <v>101698</v>
+        <v>90509</v>
       </c>
       <c r="J4" t="n">
-        <v>132986</v>
+        <v>144795</v>
       </c>
       <c r="K4" t="n">
-        <v>-31288</v>
+        <v>-54286</v>
       </c>
       <c r="L4" t="n">
-        <v>-0.23</v>
+        <v>-0.33</v>
       </c>
       <c r="M4" t="n">
-        <v>-0.48</v>
+        <v>-0.62</v>
       </c>
       <c r="N4" t="n">
-        <v>24.22</v>
+        <v>18.79</v>
       </c>
       <c r="O4" t="n">
-        <v>161.01</v>
+        <v>143.6</v>
       </c>
       <c r="P4" t="n">
-        <v>63.6</v>
+        <v>71.17</v>
       </c>
       <c r="Q4" t="n">
-        <v>27867</v>
+        <v>53925</v>
       </c>
       <c r="R4" t="n">
-        <v>5073</v>
+        <v>-4886</v>
       </c>
       <c r="S4" t="n">
-        <v>-24833</v>
+        <v>-39656</v>
       </c>
       <c r="T4" t="n">
-        <v>24405</v>
+        <v>51552</v>
       </c>
       <c r="U4" t="n">
-        <v>3462</v>
+        <v>2373</v>
       </c>
       <c r="V4" t="n">
-        <v>203</v>
+        <v>61</v>
       </c>
       <c r="W4" t="n">
-        <v>8866</v>
+        <v>10887</v>
       </c>
       <c r="X4" t="n">
-        <v>33893</v>
+        <v>36632</v>
       </c>
       <c r="Y4" t="n">
-        <v>-18629</v>
+        <v>-4263</v>
       </c>
       <c r="Z4" t="n">
-        <v>33.72</v>
+        <v>24.44</v>
       </c>
       <c r="AA4" t="n">
-        <v>95236</v>
+        <v>118788</v>
       </c>
       <c r="AB4" t="n">
-        <v>103078</v>
+        <v>130514</v>
       </c>
       <c r="AC4" t="n">
-        <v>0.26</v>
+        <v>0.27</v>
       </c>
       <c r="AD4" t="n">
-        <v>16.83</v>
+        <v>9.31</v>
       </c>
       <c r="AE4" t="n">
-        <v>21075</v>
+        <v>24701</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>45745</v>
+        <v>45836</v>
       </c>
       <c r="B5" t="n">
-        <v>164.35</v>
+        <v>140.52</v>
       </c>
       <c r="C5" t="n">
-        <v>38.86</v>
+        <v>31.43</v>
       </c>
       <c r="D5" t="n">
-        <v>2.57</v>
+        <v>3.18</v>
       </c>
       <c r="E5" t="n">
-        <v>32250</v>
+        <v>31032</v>
       </c>
       <c r="F5" t="n">
-        <v>25.99</v>
+        <v>24.92</v>
       </c>
       <c r="G5" t="n">
-        <v>61.04</v>
+        <v>49.99</v>
       </c>
       <c r="H5" t="n">
-        <v>4072542612.02</v>
+        <v>3292941690.56</v>
       </c>
       <c r="I5" t="n">
-        <v>98186</v>
+        <v>101698</v>
       </c>
       <c r="J5" t="n">
-        <v>132922</v>
+        <v>132986</v>
       </c>
       <c r="K5" t="n">
-        <v>-34736</v>
+        <v>-31288</v>
       </c>
       <c r="L5" t="n">
-        <v>-0.25</v>
+        <v>-0.23</v>
       </c>
       <c r="M5" t="n">
-        <v>-0.52</v>
+        <v>-0.48</v>
       </c>
       <c r="N5" t="n">
-        <v>29.96</v>
+        <v>24.19</v>
       </c>
       <c r="O5" t="n">
-        <v>158.98</v>
+        <v>161.01</v>
       </c>
       <c r="P5" t="n">
-        <v>64.5</v>
+        <v>63.6</v>
       </c>
       <c r="Q5" t="n">
-        <v>23952</v>
+        <v>27867</v>
       </c>
       <c r="R5" t="n">
-        <v>2917</v>
+        <v>5073</v>
       </c>
       <c r="S5" t="n">
-        <v>-29006</v>
+        <v>-24833</v>
       </c>
       <c r="T5" t="n">
-        <v>20881</v>
+        <v>24405</v>
       </c>
       <c r="U5" t="n">
-        <v>3071</v>
+        <v>3462</v>
       </c>
       <c r="V5" t="n">
-        <v>-1269</v>
+        <v>203</v>
       </c>
       <c r="W5" t="n">
-        <v>8550</v>
+        <v>8866</v>
       </c>
       <c r="X5" t="n">
-        <v>31458</v>
+        <v>33893</v>
       </c>
       <c r="Y5" t="n">
-        <v>-25897</v>
+        <v>-18629</v>
       </c>
       <c r="Z5" t="n">
-        <v>35.67</v>
+        <v>33.72</v>
       </c>
       <c r="AA5" t="n">
-        <v>86578</v>
+        <v>95236</v>
       </c>
       <c r="AB5" t="n">
-        <v>101012</v>
+        <v>103078</v>
       </c>
       <c r="AC5" t="n">
-        <v>0.25</v>
+        <v>0.26</v>
       </c>
       <c r="AD5" t="n">
-        <v>15.17</v>
+        <v>16.83</v>
       </c>
       <c r="AE5" t="n">
-        <v>25898</v>
+        <v>21075</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>45654</v>
+        <v>45745</v>
       </c>
       <c r="B6" t="n">
-        <v>86.76000000000001</v>
+        <v>164.2</v>
       </c>
       <c r="C6" t="n">
-        <v>27.76</v>
+        <v>38.82</v>
       </c>
       <c r="D6" t="n">
-        <v>3.6</v>
+        <v>2.58</v>
       </c>
       <c r="E6" t="n">
-        <v>45912</v>
+        <v>32250</v>
       </c>
       <c r="F6" t="n">
-        <v>29.23</v>
+        <v>25.99</v>
       </c>
       <c r="G6" t="n">
-        <v>47.18</v>
+        <v>60.98</v>
       </c>
       <c r="H6" t="n">
-        <v>3152080316</v>
+        <v>4068794091.52</v>
       </c>
       <c r="I6" t="n">
-        <v>96799</v>
+        <v>98186</v>
       </c>
       <c r="J6" t="n">
-        <v>141368</v>
+        <v>132922</v>
       </c>
       <c r="K6" t="n">
-        <v>-44569</v>
+        <v>-34736</v>
       </c>
       <c r="L6" t="n">
-        <v>-0.3</v>
+        <v>-0.25</v>
       </c>
       <c r="M6" t="n">
-        <v>-0.67</v>
+        <v>-0.52</v>
       </c>
       <c r="N6" t="n">
-        <v>21.59</v>
+        <v>29.93</v>
       </c>
       <c r="O6" t="n">
-        <v>172.76</v>
+        <v>158.98</v>
       </c>
       <c r="P6" t="n">
-        <v>70.51000000000001</v>
+        <v>64.5</v>
       </c>
       <c r="Q6" t="n">
-        <v>29935</v>
+        <v>23952</v>
       </c>
       <c r="R6" t="n">
-        <v>9792</v>
+        <v>2917</v>
       </c>
       <c r="S6" t="n">
-        <v>-39371</v>
+        <v>-29006</v>
       </c>
       <c r="T6" t="n">
-        <v>26995</v>
+        <v>20881</v>
       </c>
       <c r="U6" t="n">
-        <v>2940</v>
+        <v>3071</v>
       </c>
       <c r="V6" t="n">
-        <v>-2135</v>
+        <v>-1269</v>
       </c>
       <c r="W6" t="n">
-        <v>8268</v>
+        <v>8550</v>
       </c>
       <c r="X6" t="n">
-        <v>29738</v>
+        <v>31458</v>
       </c>
       <c r="Y6" t="n">
-        <v>-11125</v>
+        <v>-25897</v>
       </c>
       <c r="Z6" t="n">
-        <v>35.11</v>
+        <v>35.67</v>
       </c>
       <c r="AA6" t="n">
-        <v>87375</v>
+        <v>86578</v>
       </c>
       <c r="AB6" t="n">
-        <v>107800</v>
+        <v>101012</v>
       </c>
       <c r="AC6" t="n">
-        <v>0.26</v>
+        <v>0.25</v>
       </c>
       <c r="AD6" t="n">
-        <v>10.61</v>
+        <v>15.17</v>
       </c>
       <c r="AE6" t="n">
-        <v>23606</v>
+        <v>25898</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>45472</v>
+        <v>45654</v>
       </c>
       <c r="B7" t="n">
-        <v>121.12</v>
+        <v>86.68000000000001</v>
       </c>
       <c r="C7" t="n">
-        <v>26.59</v>
+        <v>27.73</v>
       </c>
       <c r="D7" t="n">
-        <v>3.76</v>
+        <v>3.61</v>
       </c>
       <c r="E7" t="n">
-        <v>28202</v>
+        <v>45912</v>
       </c>
       <c r="F7" t="n">
-        <v>25</v>
+        <v>29.23</v>
       </c>
       <c r="G7" t="n">
-        <v>38.97</v>
+        <v>47.14</v>
       </c>
       <c r="H7" t="n">
-        <v>2597808443.53</v>
+        <v>3149214788.44</v>
       </c>
       <c r="I7" t="n">
-        <v>101304</v>
+        <v>96799</v>
       </c>
       <c r="J7" t="n">
-        <v>153041</v>
+        <v>141368</v>
       </c>
       <c r="K7" t="n">
-        <v>-51737</v>
+        <v>-44569</v>
       </c>
       <c r="L7" t="n">
-        <v>-0.4</v>
+        <v>-0.3</v>
       </c>
       <c r="M7" t="n">
-        <v>-0.78</v>
+        <v>-0.67</v>
       </c>
       <c r="N7" t="n">
-        <v>20.67</v>
+        <v>21.57</v>
       </c>
       <c r="O7" t="n">
-        <v>148.23</v>
+        <v>172.76</v>
       </c>
       <c r="P7" t="n">
-        <v>58.86</v>
+        <v>70.51000000000001</v>
       </c>
       <c r="Q7" t="n">
-        <v>28858</v>
+        <v>29935</v>
       </c>
       <c r="R7" t="n">
-        <v>-127</v>
+        <v>9792</v>
       </c>
       <c r="S7" t="n">
-        <v>-36017</v>
+        <v>-39371</v>
       </c>
       <c r="T7" t="n">
-        <v>26707</v>
+        <v>26995</v>
       </c>
       <c r="U7" t="n">
-        <v>2151</v>
+        <v>2940</v>
       </c>
       <c r="V7" t="n">
-        <v>-2954</v>
+        <v>-2135</v>
       </c>
       <c r="W7" t="n">
-        <v>8006</v>
+        <v>8268</v>
       </c>
       <c r="X7" t="n">
-        <v>28093</v>
+        <v>29738</v>
       </c>
       <c r="Y7" t="n">
-        <v>-6189</v>
+        <v>-11125</v>
       </c>
       <c r="Z7" t="n">
-        <v>26.7</v>
+        <v>35.11</v>
       </c>
       <c r="AA7" t="n">
-        <v>92851</v>
+        <v>87375</v>
       </c>
       <c r="AB7" t="n">
-        <v>102752</v>
+        <v>107800</v>
       </c>
       <c r="AC7" t="n">
-        <v>0.25</v>
+        <v>0.26</v>
       </c>
       <c r="AD7" t="n">
-        <v>18.16</v>
+        <v>10.61</v>
       </c>
       <c r="AE7" t="n">
-        <v>26522</v>
+        <v>23606</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>45381</v>
+        <v>45472</v>
       </c>
       <c r="B8" t="n">
-        <v>162.34</v>
+        <v>121.01</v>
       </c>
       <c r="C8" t="n">
-        <v>38.2</v>
+        <v>26.57</v>
       </c>
       <c r="D8" t="n">
-        <v>2.62</v>
+        <v>3.76</v>
       </c>
       <c r="E8" t="n">
-        <v>30736</v>
+        <v>28202</v>
       </c>
       <c r="F8" t="n">
-        <v>26.04</v>
+        <v>25</v>
       </c>
       <c r="G8" t="n">
-        <v>51.67</v>
+        <v>38.94</v>
       </c>
       <c r="H8" t="n">
-        <v>3836982495.36</v>
+        <v>2595515315.38</v>
       </c>
       <c r="I8" t="n">
-        <v>104590</v>
+        <v>101304</v>
       </c>
       <c r="J8" t="n">
-        <v>162337</v>
+        <v>153041</v>
       </c>
       <c r="K8" t="n">
-        <v>-57747</v>
+        <v>-51737</v>
       </c>
       <c r="L8" t="n">
-        <v>-0.44</v>
+        <v>-0.4</v>
       </c>
       <c r="M8" t="n">
         <v>-0.78</v>
       </c>
       <c r="N8" t="n">
-        <v>29.68</v>
+        <v>20.65</v>
       </c>
       <c r="O8" t="n">
-        <v>136.93</v>
+        <v>148.23</v>
       </c>
       <c r="P8" t="n">
-        <v>56.88</v>
+        <v>58.86</v>
       </c>
       <c r="Q8" t="n">
-        <v>22690</v>
+        <v>28858</v>
       </c>
       <c r="R8" t="n">
-        <v>-310</v>
+        <v>-127</v>
       </c>
       <c r="S8" t="n">
-        <v>-30433</v>
+        <v>-36017</v>
       </c>
       <c r="T8" t="n">
-        <v>20694</v>
+        <v>26707</v>
       </c>
       <c r="U8" t="n">
-        <v>1996</v>
+        <v>2151</v>
       </c>
       <c r="V8" t="n">
-        <v>-2237</v>
+        <v>-2954</v>
       </c>
       <c r="W8" t="n">
-        <v>7903</v>
+        <v>8006</v>
       </c>
       <c r="X8" t="n">
-        <v>28261</v>
+        <v>28093</v>
       </c>
       <c r="Y8" t="n">
-        <v>4594</v>
+        <v>-6189</v>
       </c>
       <c r="Z8" t="n">
-        <v>33.46</v>
+        <v>26.7</v>
       </c>
       <c r="AA8" t="n">
-        <v>88655</v>
+        <v>92851</v>
       </c>
       <c r="AB8" t="n">
-        <v>97215</v>
+        <v>102752</v>
       </c>
       <c r="AC8" t="n">
-        <v>0.24</v>
+        <v>0.25</v>
       </c>
       <c r="AD8" t="n">
-        <v>15.7</v>
+        <v>18.16</v>
       </c>
       <c r="AE8" t="n">
-        <v>23205</v>
+        <v>26522</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>45290</v>
+        <v>45381</v>
       </c>
       <c r="B9" t="n">
-        <v>87.55</v>
+        <v>162.19</v>
       </c>
       <c r="C9" t="n">
-        <v>27.83</v>
+        <v>38.16</v>
       </c>
       <c r="D9" t="n">
-        <v>3.59</v>
+        <v>2.62</v>
       </c>
       <c r="E9" t="n">
-        <v>43221</v>
+        <v>30736</v>
       </c>
       <c r="F9" t="n">
-        <v>28.36</v>
+        <v>26.04</v>
       </c>
       <c r="G9" t="n">
-        <v>40.05</v>
+        <v>51.62</v>
       </c>
       <c r="H9" t="n">
-        <v>2969499223.98</v>
+        <v>3833439148.48</v>
       </c>
       <c r="I9" t="n">
-        <v>108040</v>
+        <v>104590</v>
       </c>
       <c r="J9" t="n">
-        <v>172575</v>
+        <v>162337</v>
       </c>
       <c r="K9" t="n">
-        <v>-64535</v>
+        <v>-57747</v>
       </c>
       <c r="L9" t="n">
-        <v>-0.46</v>
+        <v>-0.44</v>
       </c>
       <c r="M9" t="n">
-        <v>-0.87</v>
+        <v>-0.78</v>
       </c>
       <c r="N9" t="n">
-        <v>21.76</v>
+        <v>29.65</v>
       </c>
       <c r="O9" t="n">
-        <v>145.69</v>
+        <v>136.93</v>
       </c>
       <c r="P9" t="n">
-        <v>59.62</v>
+        <v>56.88</v>
       </c>
       <c r="Q9" t="n">
-        <v>39895</v>
+        <v>22690</v>
       </c>
       <c r="R9" t="n">
-        <v>1927</v>
+        <v>-310</v>
       </c>
       <c r="S9" t="n">
-        <v>-30585</v>
+        <v>-30433</v>
       </c>
       <c r="T9" t="n">
-        <v>37503</v>
+        <v>20694</v>
       </c>
       <c r="U9" t="n">
-        <v>2392</v>
+        <v>1996</v>
       </c>
       <c r="V9" t="n">
-        <v>-526</v>
+        <v>-2237</v>
       </c>
       <c r="W9" t="n">
-        <v>7696</v>
+        <v>7903</v>
       </c>
       <c r="X9" t="n">
-        <v>29778</v>
+        <v>28261</v>
       </c>
       <c r="Y9" t="n">
-        <v>9719</v>
+        <v>4594</v>
       </c>
       <c r="Z9" t="n">
-        <v>26.39</v>
+        <v>33.46</v>
       </c>
       <c r="AA9" t="n">
-        <v>93726</v>
+        <v>88655</v>
       </c>
       <c r="AB9" t="n">
-        <v>109063</v>
+        <v>97215</v>
       </c>
       <c r="AC9" t="n">
-        <v>0.25</v>
+        <v>0.24</v>
       </c>
       <c r="AD9" t="n">
-        <v>11.28</v>
+        <v>15.7</v>
       </c>
       <c r="AE9" t="n">
-        <v>20139</v>
+        <v>23205</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>45078</v>
+        <v>45290</v>
       </c>
       <c r="B10" t="n">
-        <v>128.35</v>
+        <v>87.48</v>
       </c>
       <c r="C10" t="n">
-        <v>27.6</v>
+        <v>27.8</v>
       </c>
       <c r="D10" t="n">
-        <v>3.62</v>
+        <v>3.6</v>
       </c>
       <c r="E10" t="n">
-        <v>26050</v>
+        <v>43221</v>
       </c>
       <c r="F10" t="n">
-        <v>24.31</v>
+        <v>28.36</v>
       </c>
       <c r="G10" t="n">
-        <v>42.33</v>
+        <v>40.02</v>
       </c>
       <c r="H10" t="n">
-        <v>2551647155.7</v>
+        <v>2966862564.27</v>
       </c>
       <c r="I10" t="n">
-        <v>109280</v>
+        <v>108040</v>
       </c>
       <c r="J10" t="n">
-        <v>166543</v>
+        <v>172575</v>
       </c>
       <c r="K10" t="n">
-        <v>-57263</v>
+        <v>-64535</v>
       </c>
       <c r="L10" t="n">
-        <v>-0.47</v>
+        <v>-0.46</v>
       </c>
       <c r="M10" t="n">
-        <v>-0.95</v>
+        <v>-0.87</v>
       </c>
       <c r="N10" t="n">
-        <v>21.37</v>
+        <v>21.74</v>
       </c>
       <c r="O10" t="n">
-        <v>155.09</v>
+        <v>145.69</v>
       </c>
       <c r="P10" t="n">
-        <v>55.49</v>
+        <v>59.62</v>
       </c>
       <c r="Q10" t="n">
-        <v>26380</v>
+        <v>39895</v>
       </c>
       <c r="R10" t="n">
-        <v>437</v>
+        <v>1927</v>
       </c>
       <c r="S10" t="n">
-        <v>-24048</v>
+        <v>-30585</v>
       </c>
       <c r="T10" t="n">
-        <v>24287</v>
+        <v>37503</v>
       </c>
       <c r="U10" t="n">
-        <v>2093</v>
+        <v>2392</v>
       </c>
       <c r="V10" t="n">
-        <v>-773</v>
+        <v>-526</v>
       </c>
       <c r="W10" t="n">
-        <v>7442</v>
+        <v>7696</v>
       </c>
       <c r="X10" t="n">
-        <v>28632</v>
+        <v>29778</v>
       </c>
       <c r="Y10" t="n">
-        <v>-2304</v>
+        <v>9719</v>
       </c>
       <c r="Z10" t="n">
-        <v>29.64</v>
+        <v>26.39</v>
       </c>
       <c r="AA10" t="n">
-        <v>76138</v>
+        <v>93726</v>
       </c>
       <c r="AB10" t="n">
-        <v>98079</v>
+        <v>109063</v>
       </c>
       <c r="AC10" t="n">
         <v>0.25</v>
       </c>
       <c r="AD10" t="n">
-        <v>19.36</v>
+        <v>11.28</v>
       </c>
       <c r="AE10" t="n">
-        <v>17478</v>
+        <v>20139</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>44986</v>
+        <v>45078</v>
       </c>
       <c r="B11" t="n">
-        <v>124.51</v>
+        <v>128.23</v>
       </c>
       <c r="C11" t="n">
-        <v>30.93</v>
+        <v>27.57</v>
       </c>
       <c r="D11" t="n">
-        <v>3.23</v>
+        <v>3.63</v>
       </c>
       <c r="E11" t="n">
-        <v>31216</v>
+        <v>26050</v>
       </c>
       <c r="F11" t="n">
-        <v>25.48</v>
+        <v>24.31</v>
       </c>
       <c r="G11" t="n">
-        <v>48.36</v>
+        <v>42.29</v>
       </c>
       <c r="H11" t="n">
-        <v>3008242194.7</v>
+        <v>2549292513.6</v>
       </c>
       <c r="I11" t="n">
-        <v>109615</v>
+        <v>109280</v>
       </c>
       <c r="J11" t="n">
-        <v>166333</v>
+        <v>166543</v>
       </c>
       <c r="K11" t="n">
-        <v>-56718</v>
+        <v>-57263</v>
       </c>
       <c r="L11" t="n">
-        <v>-0.44</v>
+        <v>-0.47</v>
       </c>
       <c r="M11" t="n">
-        <v>-0.91</v>
+        <v>-0.95</v>
       </c>
       <c r="N11" t="n">
-        <v>23.81</v>
+        <v>21.35</v>
       </c>
       <c r="O11" t="n">
-        <v>158.64</v>
+        <v>155.09</v>
       </c>
       <c r="P11" t="n">
-        <v>57.51</v>
+        <v>55.49</v>
       </c>
       <c r="Q11" t="n">
-        <v>28560</v>
+        <v>26380</v>
       </c>
       <c r="R11" t="n">
-        <v>2319</v>
+        <v>437</v>
       </c>
       <c r="S11" t="n">
-        <v>-25724</v>
+        <v>-24048</v>
       </c>
       <c r="T11" t="n">
-        <v>25644</v>
+        <v>24287</v>
       </c>
       <c r="U11" t="n">
-        <v>2916</v>
+        <v>2093</v>
       </c>
       <c r="V11" t="n">
-        <v>-37</v>
+        <v>-773</v>
       </c>
       <c r="W11" t="n">
-        <v>7457</v>
+        <v>7442</v>
       </c>
       <c r="X11" t="n">
-        <v>28313</v>
+        <v>28632</v>
       </c>
       <c r="Y11" t="n">
-        <v>-7162</v>
+        <v>-2304</v>
       </c>
       <c r="Z11" t="n">
-        <v>28.29</v>
+        <v>29.64</v>
       </c>
       <c r="AA11" t="n">
-        <v>76678</v>
+        <v>76138</v>
       </c>
       <c r="AB11" t="n">
-        <v>100326</v>
+        <v>98079</v>
       </c>
       <c r="AC11" t="n">
-        <v>0.23</v>
+        <v>0.25</v>
       </c>
       <c r="AD11" t="n">
-        <v>15.11</v>
+        <v>19.36</v>
       </c>
       <c r="AE11" t="n">
-        <v>19594</v>
+        <v>17478</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>44926</v>
+        <v>44986</v>
       </c>
       <c r="B12" t="n">
-        <v>71.06999999999999</v>
+        <v>124.4</v>
       </c>
       <c r="C12" t="n">
-        <v>19.9</v>
+        <v>30.91</v>
       </c>
       <c r="D12" t="n">
-        <v>5.02</v>
+        <v>3.24</v>
       </c>
       <c r="E12" t="n">
-        <v>38932</v>
+        <v>31216</v>
       </c>
       <c r="F12" t="n">
-        <v>25.61</v>
+        <v>25.48</v>
       </c>
       <c r="G12" t="n">
-        <v>37.58</v>
+        <v>48.32</v>
       </c>
       <c r="H12" t="n">
-        <v>2132008790.45</v>
+        <v>3005558378.52</v>
       </c>
       <c r="I12" t="n">
-        <v>111110</v>
+        <v>109615</v>
       </c>
       <c r="J12" t="n">
-        <v>165450</v>
+        <v>166333</v>
       </c>
       <c r="K12" t="n">
-        <v>-54340</v>
+        <v>-56718</v>
       </c>
       <c r="L12" t="n">
-        <v>-0.38</v>
+        <v>-0.44</v>
       </c>
       <c r="M12" t="n">
-        <v>-0.96</v>
+        <v>-0.91</v>
       </c>
       <c r="N12" t="n">
-        <v>15.43</v>
+        <v>23.79</v>
       </c>
       <c r="O12" t="n">
-        <v>192.29</v>
+        <v>158.64</v>
       </c>
       <c r="P12" t="n">
-        <v>65.28</v>
+        <v>57.51</v>
       </c>
       <c r="Q12" t="n">
-        <v>34005</v>
+        <v>28560</v>
       </c>
       <c r="R12" t="n">
-        <v>-1445</v>
+        <v>2319</v>
       </c>
       <c r="S12" t="n">
-        <v>-35563</v>
+        <v>-25724</v>
       </c>
       <c r="T12" t="n">
-        <v>30218</v>
+        <v>25644</v>
       </c>
       <c r="U12" t="n">
-        <v>3787</v>
+        <v>2916</v>
       </c>
       <c r="V12" t="n">
-        <v>51</v>
+        <v>-37</v>
       </c>
       <c r="W12" t="n">
-        <v>7709</v>
+        <v>7457</v>
       </c>
       <c r="X12" t="n">
-        <v>27250</v>
+        <v>28313</v>
       </c>
       <c r="Y12" t="n">
-        <v>-8509</v>
+        <v>-7162</v>
       </c>
       <c r="Z12" t="n">
-        <v>26.36</v>
+        <v>28.29</v>
       </c>
       <c r="AA12" t="n">
-        <v>86066</v>
+        <v>76678</v>
       </c>
       <c r="AB12" t="n">
-        <v>108264</v>
+        <v>100326</v>
       </c>
       <c r="AC12" t="n">
-        <v>0.24</v>
+        <v>0.23</v>
       </c>
       <c r="AD12" t="n">
-        <v>12.56</v>
+        <v>15.11</v>
       </c>
       <c r="AE12" t="n">
-        <v>19475</v>
+        <v>19594</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>44737</v>
+        <v>44926</v>
       </c>
       <c r="B13" t="n">
-        <v>142.23</v>
+        <v>71.01000000000001</v>
       </c>
       <c r="C13" t="n">
-        <v>27.77</v>
+        <v>19.89</v>
       </c>
       <c r="D13" t="n">
-        <v>3.6</v>
+        <v>5.03</v>
       </c>
       <c r="E13" t="n">
-        <v>25881</v>
+        <v>38932</v>
       </c>
       <c r="F13" t="n">
-        <v>23.44</v>
+        <v>25.61</v>
       </c>
       <c r="G13" t="n">
-        <v>47.52</v>
+        <v>37.54</v>
       </c>
       <c r="H13" t="n">
-        <v>2765156630.6</v>
+        <v>2130101663.69</v>
       </c>
       <c r="I13" t="n">
-        <v>119691</v>
+        <v>111110</v>
       </c>
       <c r="J13" t="n">
-        <v>179308</v>
+        <v>165450</v>
       </c>
       <c r="K13" t="n">
-        <v>-59617</v>
+        <v>-54340</v>
       </c>
       <c r="L13" t="n">
-        <v>-0.46</v>
+        <v>-0.38</v>
       </c>
       <c r="M13" t="n">
-        <v>-1.03</v>
+        <v>-0.96</v>
       </c>
       <c r="N13" t="n">
-        <v>21.77</v>
+        <v>15.41</v>
       </c>
       <c r="O13" t="n">
-        <v>173.52</v>
+        <v>192.29</v>
       </c>
       <c r="P13" t="n">
-        <v>56.63</v>
+        <v>65.28</v>
       </c>
       <c r="Q13" t="n">
-        <v>22892</v>
+        <v>34005</v>
       </c>
       <c r="R13" t="n">
-        <v>4234</v>
+        <v>-1445</v>
       </c>
       <c r="S13" t="n">
-        <v>-27445</v>
+        <v>-35563</v>
       </c>
       <c r="T13" t="n">
-        <v>20790</v>
+        <v>30218</v>
       </c>
       <c r="U13" t="n">
-        <v>2102</v>
+        <v>3787</v>
       </c>
       <c r="V13" t="n">
-        <v>-1559</v>
+        <v>51</v>
       </c>
       <c r="W13" t="n">
-        <v>6797</v>
+        <v>7709</v>
       </c>
       <c r="X13" t="n">
-        <v>23648</v>
+        <v>27250</v>
       </c>
       <c r="Y13" t="n">
-        <v>-17581</v>
+        <v>-8509</v>
       </c>
       <c r="Z13" t="n">
-        <v>26.33</v>
+        <v>26.36</v>
       </c>
       <c r="AA13" t="n">
-        <v>81807</v>
+        <v>86066</v>
       </c>
       <c r="AB13" t="n">
-        <v>98725</v>
+        <v>108264</v>
       </c>
       <c r="AC13" t="n">
         <v>0.24</v>
       </c>
       <c r="AD13" t="n">
-        <v>19.6</v>
+        <v>12.56</v>
       </c>
       <c r="AE13" t="n">
-        <v>21865</v>
+        <v>19475</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>44646</v>
+        <v>44737</v>
       </c>
       <c r="B14" t="n">
-        <v>83.23999999999999</v>
+        <v>142.09</v>
       </c>
       <c r="C14" t="n">
-        <v>20.08</v>
+        <v>27.75</v>
       </c>
       <c r="D14" t="n">
-        <v>4.98</v>
+        <v>3.6</v>
       </c>
       <c r="E14" t="n">
-        <v>32716</v>
+        <v>25881</v>
       </c>
       <c r="F14" t="n">
-        <v>25.71</v>
+        <v>23.44</v>
       </c>
       <c r="G14" t="n">
-        <v>30.89</v>
+        <v>47.48</v>
       </c>
       <c r="H14" t="n">
-        <v>2081733199.76</v>
+        <v>2762570559.4</v>
       </c>
       <c r="I14" t="n">
-        <v>119981</v>
+        <v>119691</v>
       </c>
       <c r="J14" t="n">
-        <v>192730</v>
+        <v>179308</v>
       </c>
       <c r="K14" t="n">
-        <v>-72749</v>
+        <v>-59617</v>
       </c>
       <c r="L14" t="n">
-        <v>-0.54</v>
+        <v>-0.46</v>
       </c>
       <c r="M14" t="n">
-        <v>-1.08</v>
+        <v>-1.03</v>
       </c>
       <c r="N14" t="n">
-        <v>16.06</v>
+        <v>21.75</v>
       </c>
       <c r="O14" t="n">
-        <v>155.81</v>
+        <v>173.52</v>
       </c>
       <c r="P14" t="n">
-        <v>55.69</v>
+        <v>56.63</v>
       </c>
       <c r="Q14" t="n">
-        <v>28166</v>
+        <v>22892</v>
       </c>
       <c r="R14" t="n">
-        <v>-9265</v>
+        <v>4234</v>
       </c>
       <c r="S14" t="n">
-        <v>-28351</v>
+        <v>-27445</v>
       </c>
       <c r="T14" t="n">
-        <v>25652</v>
+        <v>20790</v>
       </c>
       <c r="U14" t="n">
-        <v>2514</v>
+        <v>2102</v>
       </c>
       <c r="V14" t="n">
-        <v>-1384</v>
+        <v>-1559</v>
       </c>
       <c r="W14" t="n">
-        <v>6387</v>
+        <v>6797</v>
       </c>
       <c r="X14" t="n">
-        <v>22288</v>
+        <v>23648</v>
       </c>
       <c r="Y14" t="n">
-        <v>-9328</v>
+        <v>-17581</v>
       </c>
       <c r="Z14" t="n">
-        <v>23.48</v>
+        <v>26.33</v>
       </c>
       <c r="AA14" t="n">
-        <v>103855</v>
+        <v>81807</v>
       </c>
       <c r="AB14" t="n">
-        <v>101315</v>
+        <v>98725</v>
       </c>
       <c r="AC14" t="n">
-        <v>0.22</v>
+        <v>0.24</v>
       </c>
       <c r="AD14" t="n">
-        <v>14.37</v>
+        <v>19.6</v>
       </c>
       <c r="AE14" t="n">
-        <v>22631</v>
+        <v>21865</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>44555</v>
+        <v>44646</v>
       </c>
       <c r="B15" t="n">
-        <v>63.25</v>
+        <v>83.16</v>
       </c>
       <c r="C15" t="n">
-        <v>20.46</v>
+        <v>20.06</v>
       </c>
       <c r="D15" t="n">
-        <v>4.89</v>
+        <v>4.99</v>
       </c>
       <c r="E15" t="n">
-        <v>44185</v>
+        <v>32716</v>
       </c>
       <c r="F15" t="n">
-        <v>27.94</v>
+        <v>25.71</v>
       </c>
       <c r="G15" t="n">
-        <v>30.44</v>
+        <v>30.86</v>
       </c>
       <c r="H15" t="n">
-        <v>2190426078.12</v>
+        <v>2079779743.52</v>
       </c>
       <c r="I15" t="n">
-        <v>122798</v>
+        <v>119981</v>
       </c>
       <c r="J15" t="n">
-        <v>202596</v>
+        <v>192730</v>
       </c>
       <c r="K15" t="n">
-        <v>-79798</v>
+        <v>-72749</v>
       </c>
       <c r="L15" t="n">
-        <v>-0.58</v>
+        <v>-0.54</v>
       </c>
       <c r="M15" t="n">
-        <v>-1.11</v>
+        <v>-1.08</v>
       </c>
       <c r="N15" t="n">
-        <v>16.49</v>
+        <v>16.04</v>
       </c>
       <c r="O15" t="n">
-        <v>151.2</v>
+        <v>155.81</v>
       </c>
       <c r="P15" t="n">
-        <v>55.57</v>
+        <v>55.69</v>
       </c>
       <c r="Q15" t="n">
-        <v>46966</v>
+        <v>28166</v>
       </c>
       <c r="R15" t="n">
-        <v>-16106</v>
+        <v>-9265</v>
       </c>
       <c r="S15" t="n">
-        <v>-28159</v>
+        <v>-28351</v>
       </c>
       <c r="T15" t="n">
-        <v>44163</v>
+        <v>25652</v>
       </c>
       <c r="U15" t="n">
-        <v>2803</v>
+        <v>2514</v>
       </c>
       <c r="V15" t="n">
-        <v>-327</v>
+        <v>-1384</v>
       </c>
       <c r="W15" t="n">
-        <v>6306</v>
+        <v>6387</v>
       </c>
       <c r="X15" t="n">
-        <v>22121</v>
+        <v>22288</v>
       </c>
       <c r="Y15" t="n">
-        <v>5580</v>
+        <v>-9328</v>
       </c>
       <c r="Z15" t="n">
-        <v>14.84</v>
+        <v>23.48</v>
       </c>
       <c r="AA15" t="n">
-        <v>117550</v>
+        <v>103855</v>
       </c>
       <c r="AB15" t="n">
-        <v>112739</v>
+        <v>101315</v>
       </c>
       <c r="AC15" t="n">
-        <v>0.23</v>
+        <v>0.22</v>
       </c>
       <c r="AD15" t="n">
-        <v>10.78</v>
+        <v>14.37</v>
       </c>
       <c r="AE15" t="n">
-        <v>20478</v>
+        <v>22631</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>44373</v>
+        <v>44555</v>
       </c>
       <c r="B16" t="n">
-        <v>90.98999999999999</v>
+        <v>63.19</v>
       </c>
       <c r="C16" t="n">
-        <v>16.92</v>
+        <v>20.44</v>
       </c>
       <c r="D16" t="n">
-        <v>5.91</v>
+        <v>4.89</v>
       </c>
       <c r="E16" t="n">
-        <v>26958</v>
+        <v>44185</v>
       </c>
       <c r="F16" t="n">
-        <v>26.7</v>
+        <v>27.94</v>
       </c>
       <c r="G16" t="n">
-        <v>30.74</v>
+        <v>30.41</v>
       </c>
       <c r="H16" t="n">
-        <v>1978396267.87</v>
+        <v>2188295154</v>
       </c>
       <c r="I16" t="n">
-        <v>121791</v>
+        <v>122798</v>
       </c>
       <c r="J16" t="n">
-        <v>193644</v>
+        <v>202596</v>
       </c>
       <c r="K16" t="n">
-        <v>-71853</v>
+        <v>-79798</v>
       </c>
       <c r="L16" t="n">
-        <v>-0.66</v>
+        <v>-0.58</v>
       </c>
       <c r="M16" t="n">
-        <v>-1.12</v>
+        <v>-1.11</v>
       </c>
       <c r="N16" t="n">
-        <v>18.76</v>
+        <v>16.48</v>
       </c>
       <c r="O16" t="n">
-        <v>132.83</v>
+        <v>151.2</v>
       </c>
       <c r="P16" t="n">
-        <v>45.43</v>
+        <v>55.57</v>
       </c>
       <c r="Q16" t="n">
-        <v>21094</v>
+        <v>46966</v>
       </c>
       <c r="R16" t="n">
-        <v>3572</v>
+        <v>-16106</v>
       </c>
       <c r="S16" t="n">
-        <v>-29396</v>
+        <v>-28159</v>
       </c>
       <c r="T16" t="n">
-        <v>19001</v>
+        <v>44163</v>
       </c>
       <c r="U16" t="n">
-        <v>2093</v>
+        <v>2803</v>
       </c>
       <c r="V16" t="n">
-        <v>-1620</v>
+        <v>-327</v>
       </c>
       <c r="W16" t="n">
-        <v>5717</v>
+        <v>6306</v>
       </c>
       <c r="X16" t="n">
-        <v>19280</v>
+        <v>22121</v>
       </c>
       <c r="Y16" t="n">
-        <v>6669</v>
+        <v>5580</v>
       </c>
       <c r="Z16" t="n">
-        <v>28.48</v>
+        <v>14.84</v>
       </c>
       <c r="AA16" t="n">
-        <v>88143</v>
+        <v>117550</v>
       </c>
       <c r="AB16" t="n">
-        <v>84497</v>
+        <v>112739</v>
       </c>
       <c r="AC16" t="n">
         <v>0.23</v>
       </c>
       <c r="AD16" t="n">
-        <v>17.32</v>
+        <v>10.78</v>
       </c>
       <c r="AE16" t="n">
-        <v>22900</v>
+        <v>20478</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>44282</v>
+        <v>44373</v>
       </c>
       <c r="B17" t="n">
-        <v>123.19</v>
+        <v>90.90000000000001</v>
       </c>
       <c r="C17" t="n">
-        <v>20.93</v>
+        <v>16.91</v>
       </c>
       <c r="D17" t="n">
-        <v>4.78</v>
+        <v>5.91</v>
       </c>
       <c r="E17" t="n">
-        <v>30300</v>
+        <v>26958</v>
       </c>
       <c r="F17" t="n">
-        <v>26.38</v>
+        <v>26.7</v>
       </c>
       <c r="G17" t="n">
-        <v>42.07</v>
+        <v>30.71</v>
       </c>
       <c r="H17" t="n">
-        <v>2911083989.76</v>
+        <v>1976567037.06</v>
       </c>
       <c r="I17" t="n">
-        <v>121645</v>
+        <v>121791</v>
       </c>
       <c r="J17" t="n">
-        <v>204373</v>
+        <v>193644</v>
       </c>
       <c r="K17" t="n">
-        <v>-82728</v>
+        <v>-71853</v>
       </c>
       <c r="L17" t="n">
-        <v>-0.84</v>
+        <v>-0.66</v>
       </c>
       <c r="M17" t="n">
-        <v>-1.2</v>
+        <v>-1.12</v>
       </c>
       <c r="N17" t="n">
-        <v>30.55</v>
+        <v>18.74</v>
       </c>
       <c r="O17" t="n">
-        <v>108.25</v>
+        <v>132.83</v>
       </c>
       <c r="P17" t="n">
-        <v>38.78</v>
+        <v>45.43</v>
       </c>
       <c r="Q17" t="n">
-        <v>23981</v>
+        <v>21094</v>
       </c>
       <c r="R17" t="n">
-        <v>-10368</v>
+        <v>3572</v>
       </c>
       <c r="S17" t="n">
-        <v>-11326</v>
+        <v>-29396</v>
       </c>
       <c r="T17" t="n">
-        <v>21712</v>
+        <v>19001</v>
       </c>
       <c r="U17" t="n">
-        <v>2269</v>
+        <v>2093</v>
       </c>
       <c r="V17" t="n">
-        <v>-1814</v>
+        <v>-1620</v>
       </c>
       <c r="W17" t="n">
-        <v>5262</v>
+        <v>5717</v>
       </c>
       <c r="X17" t="n">
-        <v>17934</v>
+        <v>19280</v>
       </c>
       <c r="Y17" t="n">
-        <v>15080</v>
+        <v>6669</v>
       </c>
       <c r="Z17" t="n">
-        <v>29.75</v>
+        <v>28.48</v>
       </c>
       <c r="AA17" t="n">
-        <v>79766</v>
+        <v>88143</v>
       </c>
       <c r="AB17" t="n">
-        <v>71111</v>
+        <v>84497</v>
       </c>
       <c r="AC17" t="n">
-        <v>0.21</v>
+        <v>0.23</v>
       </c>
       <c r="AD17" t="n">
-        <v>14.59</v>
+        <v>17.32</v>
       </c>
       <c r="AE17" t="n">
-        <v>18548</v>
+        <v>22900</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>44191</v>
+        <v>44282</v>
       </c>
       <c r="B18" t="n">
-        <v>76</v>
+        <v>123.08</v>
       </c>
       <c r="C18" t="n">
-        <v>10.82</v>
+        <v>20.92</v>
       </c>
       <c r="D18" t="n">
-        <v>9.24</v>
+        <v>4.78</v>
       </c>
       <c r="E18" t="n">
-        <v>36200</v>
+        <v>30300</v>
       </c>
       <c r="F18" t="n">
-        <v>25.8</v>
+        <v>26.38</v>
       </c>
       <c r="G18" t="n">
-        <v>33.01</v>
+        <v>42.03</v>
       </c>
       <c r="H18" t="n">
-        <v>2185477106.95</v>
+        <v>2908403433.6</v>
       </c>
       <c r="I18" t="n">
-        <v>112043</v>
+        <v>121645</v>
       </c>
       <c r="J18" t="n">
-        <v>195571</v>
+        <v>204373</v>
       </c>
       <c r="K18" t="n">
-        <v>-83528</v>
+        <v>-82728</v>
       </c>
       <c r="L18" t="n">
-        <v>-0.87</v>
+        <v>-0.84</v>
       </c>
       <c r="M18" t="n">
-        <v>-1.26</v>
+        <v>-1.2</v>
       </c>
       <c r="N18" t="n">
-        <v>23.62</v>
+        <v>30.53</v>
       </c>
       <c r="O18" t="n">
-        <v>110.98</v>
+        <v>108.25</v>
       </c>
       <c r="P18" t="n">
-        <v>40.82</v>
+        <v>38.78</v>
       </c>
       <c r="Q18" t="n">
-        <v>38763</v>
+        <v>23981</v>
       </c>
       <c r="R18" t="n">
-        <v>-8584</v>
+        <v>-10368</v>
       </c>
       <c r="S18" t="n">
-        <v>-32249</v>
+        <v>-11326</v>
       </c>
       <c r="T18" t="n">
-        <v>35263</v>
+        <v>21712</v>
       </c>
       <c r="U18" t="n">
-        <v>3500</v>
+        <v>2269</v>
       </c>
       <c r="V18" t="n">
-        <v>-1995</v>
+        <v>-1814</v>
       </c>
       <c r="W18" t="n">
-        <v>5163</v>
+        <v>5262</v>
       </c>
       <c r="X18" t="n">
-        <v>16942</v>
+        <v>17934</v>
       </c>
       <c r="Y18" t="n">
-        <v>21599</v>
+        <v>15080</v>
       </c>
       <c r="Z18" t="n">
-        <v>17.77</v>
+        <v>29.75</v>
       </c>
       <c r="AA18" t="n">
-        <v>76455</v>
+        <v>79766</v>
       </c>
       <c r="AB18" t="n">
-        <v>78838</v>
+        <v>71111</v>
       </c>
       <c r="AC18" t="n">
         <v>0.21</v>
       </c>
       <c r="AD18" t="n">
+        <v>14.59</v>
+      </c>
+      <c r="AE18" t="n">
+        <v>18548</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>44191</v>
+      </c>
+      <c r="B19" t="n">
+        <v>75.93000000000001</v>
+      </c>
+      <c r="C19" t="n">
+        <v>10.81</v>
+      </c>
+      <c r="D19" t="n">
+        <v>9.25</v>
+      </c>
+      <c r="E19" t="n">
+        <v>36200</v>
+      </c>
+      <c r="F19" t="n">
+        <v>25.8</v>
+      </c>
+      <c r="G19" t="n">
+        <v>32.97</v>
+      </c>
+      <c r="H19" t="n">
+        <v>2183444892.67</v>
+      </c>
+      <c r="I19" t="n">
+        <v>112043</v>
+      </c>
+      <c r="J19" t="n">
+        <v>195571</v>
+      </c>
+      <c r="K19" t="n">
+        <v>-83528</v>
+      </c>
+      <c r="L19" t="n">
+        <v>-0.87</v>
+      </c>
+      <c r="M19" t="n">
+        <v>-1.26</v>
+      </c>
+      <c r="N19" t="n">
+        <v>23.6</v>
+      </c>
+      <c r="O19" t="n">
+        <v>110.98</v>
+      </c>
+      <c r="P19" t="n">
+        <v>40.82</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>38763</v>
+      </c>
+      <c r="R19" t="n">
+        <v>-8584</v>
+      </c>
+      <c r="S19" t="n">
+        <v>-32249</v>
+      </c>
+      <c r="T19" t="n">
+        <v>35263</v>
+      </c>
+      <c r="U19" t="n">
+        <v>3500</v>
+      </c>
+      <c r="V19" t="n">
+        <v>-1995</v>
+      </c>
+      <c r="W19" t="n">
+        <v>5163</v>
+      </c>
+      <c r="X19" t="n">
+        <v>16942</v>
+      </c>
+      <c r="Y19" t="n">
+        <v>21599</v>
+      </c>
+      <c r="Z19" t="n">
+        <v>17.77</v>
+      </c>
+      <c r="AA19" t="n">
+        <v>76455</v>
+      </c>
+      <c r="AB19" t="n">
+        <v>78838</v>
+      </c>
+      <c r="AC19" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="AD19" t="n">
         <v>12.56</v>
       </c>
-      <c r="AE18" t="n">
+      <c r="AE19" t="n">
         <v>24775</v>
       </c>
     </row>

</xml_diff>